<commit_message>
regenerate content from xlsx
</commit_message>
<xml_diff>
--- a/tools/content_template.xlsx
+++ b/tools/content_template.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13392" tabRatio="600" firstSheet="2" activeTab="11" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_readme" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-04_haus" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -48,13 +47,13 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -67,22 +66,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
+        <fgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001565C0"/>
+        <fgColor rgb="FF1565C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
+        <fgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006A1B9A"/>
+        <fgColor rgb="FF6A1B9A"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,17 +95,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -142,7 +142,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -506,12 +506,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Anleitung</t>
@@ -519,7 +519,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -591,21 +591,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Wochentage &amp; Tageszeiten</t>
@@ -624,7 +622,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -683,7 +681,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -735,7 +733,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.lunedi</t>
@@ -761,17 +759,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.martedi</t>
@@ -797,17 +795,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.mercoledi</t>
@@ -833,17 +831,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.giovedi</t>
@@ -869,17 +867,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.venerdi</t>
@@ -905,17 +903,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.sabato</t>
@@ -941,17 +939,17 @@
           <t>il</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.domenica</t>
@@ -977,17 +975,17 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.oggi</t>
@@ -1008,8 +1006,8 @@
           <t>adv</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Oggi è lunedì.</t>
@@ -1020,14 +1018,14 @@
           <t>Heute ist Montag.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.domani</t>
@@ -1048,8 +1046,8 @@
           <t>adv</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="inlineStr">
         <is>
           <t>A domani!</t>
@@ -1060,14 +1058,14 @@
           <t>Bis morgen!</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.ieri</t>
@@ -1088,42 +1086,98 @@
           <t>adv</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+    <row r="17" ht="28.05" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>vocab.dopodomani</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>dopodomani</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>übermorgen</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>adv</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>A dopodomani!</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Bis übermorgen!</t>
+        </is>
+      </c>
       <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>typing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28.05" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>vocab.altroieri</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>l'altroieri</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>vorgestern</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>adv</t>
+        </is>
+      </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>L'altroieri ho visto Marco.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Vorgestern habe ich Marco gesehen.</t>
+        </is>
+      </c>
       <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="28" customHeight="1">
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>typing</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -1135,7 +1189,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -1147,7 +1201,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -1188,7 +1242,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Oggi è venerdì.</t>
@@ -1199,9 +1253,9 @@
           <t>Heute ist Freitag.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Domani è sabato.</t>
@@ -1212,9 +1266,9 @@
           <t>Morgen ist Samstag.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Ci vediamo lunedì!</t>
@@ -1225,14 +1279,14 @@
           <t>Wir sehen uns am Montag!</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -1249,21 +1303,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Häufige Verben</t>
@@ -1282,7 +1334,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -1341,7 +1393,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -1393,7 +1445,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.essere</t>
@@ -1414,8 +1466,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Io sono Marco.</t>
@@ -1437,7 +1489,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.avere</t>
@@ -1458,8 +1510,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Ho fame.</t>
@@ -1481,7 +1533,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.fare</t>
@@ -1502,8 +1554,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Cosa fai?</t>
@@ -1514,14 +1566,14 @@
           <t>Was machst du?</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.andare</t>
@@ -1542,8 +1594,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Vado a casa.</t>
@@ -1554,14 +1606,14 @@
           <t>Ich gehe nach Hause.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.venire</t>
@@ -1582,8 +1634,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Vieni qui!</t>
@@ -1594,14 +1646,14 @@
           <t>Komm her!</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.mangiare</t>
@@ -1622,8 +1674,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Mangio pizza.</t>
@@ -1634,14 +1686,14 @@
           <t>Ich esse Pizza.</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.bere</t>
@@ -1662,8 +1714,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Bevo acqua.</t>
@@ -1674,14 +1726,14 @@
           <t>Ich trinke Wasser.</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.parlare</t>
@@ -1694,7 +1746,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>sprechen</t>
+          <t>sprechen/reden</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1702,8 +1754,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Parlo italiano.</t>
@@ -1714,14 +1766,14 @@
           <t>Ich spreche Italienisch.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.vedere</t>
@@ -1742,8 +1794,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Ti vedo!</t>
@@ -1754,14 +1806,14 @@
           <t>Ich sehe dich!</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.sapere</t>
@@ -1782,8 +1834,8 @@
           <t>verb</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
           <t>Non lo so.</t>
@@ -1794,50 +1846,146 @@
           <t>Ich weiß es nicht.</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+    <row r="17" ht="28.05" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>vocab.potere</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>potere</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>können / dürfen</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Posso usare il tuo telefono?</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Darf ich dein Handy nutzen?</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Modalverb (Erlaubnis/Möglichkeit)</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>typing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28.05" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>vocab.dovere</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>dovere</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>müssen</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Devo studiare per il compito in classe di domani.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Ich muss für die Klassenarbeit morgen lernen.</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Modalverb</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>typing</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28.05" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>vocab.riuscire</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>riuscire</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>schaffen / können (etw. gelingt)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-    </row>
-    <row r="20" ht="28" customHeight="1">
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Non riesco a dormire</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Ich kann nicht schlafen</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>riuscire a + Inf.</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>typing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -1849,7 +1997,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -1890,7 +2038,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Sono italiano e parlo tedesco.</t>
@@ -1901,9 +2049,9 @@
           <t>Ich bin Italiener und spreche Deutsch.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Vado a mangiare una pizza.</t>
@@ -1914,9 +2062,9 @@
           <t>Ich gehe eine Pizza essen.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Vieni a casa mia domani?</t>
@@ -1927,14 +2075,14 @@
           <t>Kommst du morgen zu mir nach Hause?</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -1951,21 +2099,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Im Haus</t>
@@ -1984,7 +2130,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -2043,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -2095,7 +2241,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.casa</t>
@@ -2136,14 +2282,14 @@
           <t>Ich gehe nach Hause.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.porta</t>
@@ -2174,16 +2320,16 @@
           <t>porte</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.finestra</t>
@@ -2214,16 +2360,16 @@
           <t>finestre</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.stanza</t>
@@ -2254,16 +2400,16 @@
           <t>stanze</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.cucina</t>
@@ -2294,16 +2440,16 @@
           <t>cucine</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.bagno</t>
@@ -2334,16 +2480,16 @@
           <t>bagni</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.letto</t>
@@ -2374,16 +2520,16 @@
           <t>letti</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.tavolo</t>
@@ -2414,16 +2560,16 @@
           <t>tavoli</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.sedia</t>
@@ -2454,16 +2600,16 @@
           <t>sedie</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.divano</t>
@@ -2494,16 +2640,16 @@
           <t>divani</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -2515,7 +2661,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -2527,7 +2673,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -2539,7 +2685,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -2551,7 +2697,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -2592,7 +2738,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>La cucina è grande.</t>
@@ -2603,9 +2749,9 @@
           <t>Die Küche ist groß.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>C'è un tavolo e quattro sedie.</t>
@@ -2616,9 +2762,9 @@
           <t>Es gibt einen Tisch und vier Stühle.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Apri la finestra, per favore.</t>
@@ -2629,14 +2775,14 @@
           <t>Öffne das Fenster, bitte.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -2653,7 +2799,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -2662,7 +2808,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Manifest</t>
@@ -2676,7 +2822,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>CHAPTERS</t>
@@ -2760,7 +2906,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="17.4" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>LESSONS</t>
@@ -3056,21 +3202,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Begrüßungen</t>
@@ -3089,7 +3233,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -3148,7 +3292,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -3200,7 +3344,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.ciao</t>
@@ -3221,8 +3365,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Ciao Marco!</t>
@@ -3233,14 +3377,14 @@
           <t>Hallo Marco!</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.buongiorno</t>
@@ -3261,8 +3405,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Buongiorno, signora.</t>
@@ -3273,14 +3417,14 @@
           <t>Guten Morgen, Frau.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.buonasera</t>
@@ -3301,8 +3445,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Buonasera a tutti!</t>
@@ -3313,14 +3457,14 @@
           <t>Guten Abend zusammen!</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.buonanotte</t>
@@ -3341,8 +3485,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Buonanotte, mamma.</t>
@@ -3353,14 +3497,14 @@
           <t>Gute Nacht, Mama.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.arrivederci</t>
@@ -3381,18 +3525,18 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.grazie</t>
@@ -3413,8 +3557,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Grazie mille!</t>
@@ -3425,14 +3569,14 @@
           <t>Vielen Dank!</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.prego</t>
@@ -3453,18 +3597,18 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.scusa</t>
@@ -3485,8 +3629,8 @@
           <t>interj</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Scusa, non ho capito.</t>
@@ -3497,14 +3641,14 @@
           <t>Entschuldige, ich habe nicht verstanden.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.si</t>
@@ -3525,18 +3669,18 @@
           <t>adv</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.no</t>
@@ -3557,18 +3701,18 @@
           <t>adv</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -3580,7 +3724,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -3592,7 +3736,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -3604,7 +3748,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -3616,7 +3760,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -3657,7 +3801,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Ciao, mi chiamo Marco.</t>
@@ -3668,9 +3812,9 @@
           <t>Hallo, ich heiße Marco.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Buongiorno! Come stai?</t>
@@ -3678,12 +3822,12 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Guten Morgen! Wie geht's?</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+          <t>Guten Morgen! Wie geht's dir?</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Grazie e arrivederci.</t>
@@ -3694,14 +3838,14 @@
           <t>Danke und auf Wiedersehen.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -3718,21 +3862,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Zahlen 1–10</t>
@@ -3751,7 +3893,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -3810,7 +3952,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -3862,7 +4004,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.uno</t>
@@ -3883,8 +4025,8 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Ho un cane.</t>
@@ -3895,14 +4037,14 @@
           <t>Ich habe einen Hund.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.due</t>
@@ -3923,8 +4065,8 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Due caffè, per favore.</t>
@@ -3932,17 +4074,17 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Zwei Kaffee, bitte.</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+          <t>Zwei Espresso, bitte.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.tre</t>
@@ -3963,8 +4105,8 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Ho tre fratelli.</t>
@@ -3975,14 +4117,14 @@
           <t>Ich habe drei Brüder.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.quattro</t>
@@ -4003,18 +4145,18 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.cinque</t>
@@ -4035,18 +4177,18 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.sei</t>
@@ -4067,10 +4209,10 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="inlineStr">
         <is>
           <t>auch 'tu sei' = du bist</t>
@@ -4082,7 +4224,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.sette</t>
@@ -4103,18 +4245,18 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.otto</t>
@@ -4135,18 +4277,18 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.nove</t>
@@ -4167,18 +4309,18 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.dieci</t>
@@ -4199,8 +4341,8 @@
           <t>num</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
           <t>Ho dieci anni.</t>
@@ -4211,14 +4353,14 @@
           <t>Ich bin zehn Jahre alt.</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -4230,7 +4372,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -4242,7 +4384,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -4254,7 +4396,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -4266,7 +4408,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -4307,7 +4449,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Ho tre mele.</t>
@@ -4318,9 +4460,9 @@
           <t>Ich habe drei Äpfel.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Uno, due, tre, quattro.</t>
@@ -4331,9 +4473,9 @@
           <t>Eins, zwei, drei, vier.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Sono le otto.</t>
@@ -4344,14 +4486,14 @@
           <t>Es ist acht Uhr.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -4368,21 +4510,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Familie</t>
@@ -4401,7 +4541,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -4460,7 +4600,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -4512,7 +4652,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.madre</t>
@@ -4553,14 +4693,14 @@
           <t>Meine Mutter ist Italienerin.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.padre</t>
@@ -4601,14 +4741,14 @@
           <t>Mein Vater arbeitet in Rom.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.fratello</t>
@@ -4639,16 +4779,16 @@
           <t>fratelli</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.sorella</t>
@@ -4679,16 +4819,16 @@
           <t>sorelle</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.figlio</t>
@@ -4719,16 +4859,16 @@
           <t>figli</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.figlia</t>
@@ -4759,16 +4899,16 @@
           <t>figlie</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.nonno</t>
@@ -4799,16 +4939,16 @@
           <t>nonni</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.nonna</t>
@@ -4839,16 +4979,16 @@
           <t>nonne</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.zio</t>
@@ -4879,16 +5019,16 @@
           <t>zii</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.zia</t>
@@ -4919,16 +5059,16 @@
           <t>zie</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -4940,7 +5080,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -4952,7 +5092,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -4964,7 +5104,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -4976,7 +5116,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -5017,7 +5157,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Mia madre è simpatica.</t>
@@ -5028,9 +5168,9 @@
           <t>Meine Mutter ist nett.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Ho un fratello e una sorella.</t>
@@ -5041,9 +5181,9 @@
           <t>Ich habe einen Bruder und eine Schwester.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Mio padre lavora a Roma.</t>
@@ -5054,14 +5194,14 @@
           <t>Mein Vater arbeitet in Rom.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -5078,21 +5218,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Adjektive</t>
@@ -5111,7 +5249,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -5170,7 +5308,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -5222,7 +5360,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.grande</t>
@@ -5243,8 +5381,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Una casa grande.</t>
@@ -5255,14 +5393,14 @@
           <t>Ein großes Haus.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.piccolo</t>
@@ -5283,8 +5421,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Un cane piccolo.</t>
@@ -5295,14 +5433,14 @@
           <t>Ein kleiner Hund.</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.bello</t>
@@ -5323,8 +5461,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Che bello!</t>
@@ -5335,14 +5473,14 @@
           <t>Wie schön!</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.brutto</t>
@@ -5363,18 +5501,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.buono</t>
@@ -5395,8 +5533,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
           <t>La pizza è buona.</t>
@@ -5407,14 +5545,14 @@
           <t>Die Pizza ist lecker.</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.cattivo</t>
@@ -5435,18 +5573,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.nuovo</t>
@@ -5467,18 +5605,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.vecchio</t>
@@ -5499,18 +5637,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.alto</t>
@@ -5531,18 +5669,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.basso</t>
@@ -5563,18 +5701,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -5586,7 +5724,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -5598,7 +5736,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -5610,7 +5748,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -5622,7 +5760,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -5663,7 +5801,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>La casa è grande e bella.</t>
@@ -5674,9 +5812,9 @@
           <t>Das Haus ist groß und schön.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Il caffè è molto buono.</t>
@@ -5687,9 +5825,9 @@
           <t>Der Kaffee ist sehr gut.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Marco è alto e Anna è bassa.</t>
@@ -5700,14 +5838,14 @@
           <t>Marco ist groß und Anna ist klein.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -5724,21 +5862,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Essen</t>
@@ -5757,7 +5893,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -5816,7 +5952,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -5868,7 +6004,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.pane</t>
@@ -5909,14 +6045,14 @@
           <t>Ich möchte Brot.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.acqua</t>
@@ -5949,22 +6085,22 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Un'acqua, per favore.</t>
+          <t>Un bicchiere d'acqua, per favore.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Ein Wasser, bitte.</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+          <t>Ein Glas Wasser, bitte.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.formaggio</t>
@@ -5995,16 +6131,16 @@
           <t>formaggi</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.pasta</t>
@@ -6035,16 +6171,16 @@
           <t>paste</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.pizza</t>
@@ -6075,16 +6211,16 @@
           <t>pizze</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.pomodoro</t>
@@ -6115,16 +6251,16 @@
           <t>pomodori</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.mela</t>
@@ -6155,16 +6291,16 @@
           <t>mele</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.frutta</t>
@@ -6190,9 +6326,9 @@
           <t>la</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="inlineStr">
         <is>
           <t>kein Plural üblich</t>
@@ -6204,7 +6340,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.verdura</t>
@@ -6235,16 +6371,16 @@
           <t>verdure</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.carne</t>
@@ -6275,16 +6411,16 @@
           <t>carni</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -6296,7 +6432,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -6308,7 +6444,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -6320,7 +6456,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -6332,7 +6468,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -6373,7 +6509,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Voglio una pizza e un'acqua.</t>
@@ -6384,9 +6520,9 @@
           <t>Ich möchte eine Pizza und ein Wasser.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Mi piace la pasta al pomodoro.</t>
@@ -6397,9 +6533,9 @@
           <t>Ich mag Tomaten-Pasta.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Ho fame, mangio del pane.</t>
@@ -6410,14 +6546,14 @@
           <t>Ich habe Hunger, ich esse Brot.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -6434,21 +6570,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Im Café</t>
@@ -6467,7 +6601,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -6526,7 +6660,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -6578,7 +6712,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.caffe</t>
@@ -6619,14 +6753,14 @@
           <t>Einen Kaffee, bitte.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.cappuccino</t>
@@ -6657,16 +6791,16 @@
           <t>cappuccini</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.te</t>
@@ -6697,16 +6831,16 @@
           <t>tè</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.latte</t>
@@ -6754,7 +6888,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.zucchero</t>
@@ -6780,17 +6914,21 @@
           <t>lo</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>zuccheri</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.biscotto</t>
@@ -6821,16 +6959,16 @@
           <t>biscotti</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.cornetto</t>
@@ -6861,16 +6999,16 @@
           <t>cornetti</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.conto</t>
@@ -6911,14 +7049,14 @@
           <t>Die Rechnung, bitte.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.cameriere</t>
@@ -6949,16 +7087,16 @@
           <t>camerieri</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.menu</t>
@@ -6989,8 +7127,8 @@
           <t>menu</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
           <t>unveränderlich</t>
@@ -7002,7 +7140,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -7014,7 +7152,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -7026,7 +7164,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -7038,7 +7176,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -7050,7 +7188,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -7091,7 +7229,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Un caffè e un cornetto, per favore.</t>
@@ -7102,12 +7240,12 @@
           <t>Einen Kaffee und ein Croissant, bitte.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Vorrei vedere il menu.</t>
+          <t>Potrei avere il menù, per favore.</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -7115,9 +7253,9 @@
           <t>Ich möchte die Speisekarte sehen.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Il conto, per favore!</t>
@@ -7128,14 +7266,14 @@
           <t>Die Rechnung, bitte!</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
@@ -7152,21 +7290,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.4" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Farben</t>
@@ -7185,7 +7321,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17.4" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>VOKABELN</t>
@@ -7244,7 +7380,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="45.6" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>z. B. vocab.ciao (stabil, nicht ändern)</t>
@@ -7296,7 +7432,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>vocab.rosso</t>
@@ -7317,8 +7453,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Una mela rossa.</t>
@@ -7329,14 +7465,14 @@
           <t>Ein roter Apfel.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>vocab.blu</t>
@@ -7357,8 +7493,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Il cielo è blu.</t>
@@ -7380,7 +7516,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>vocab.verde</t>
@@ -7401,8 +7537,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>L'erba è verde.</t>
@@ -7413,14 +7549,14 @@
           <t>Das Gras ist grün.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>vocab.giallo</t>
@@ -7441,18 +7577,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>pair</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>vocab.bianco</t>
@@ -7473,8 +7609,8 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Vino bianco.</t>
@@ -7485,14 +7621,14 @@
           <t>Weißwein.</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>vocab.nero</t>
@@ -7513,18 +7649,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="28.05" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>vocab.grigio</t>
@@ -7545,18 +7681,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>mc</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="28.05" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>vocab.marrone</t>
@@ -7577,18 +7713,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="28.05" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>vocab.arancione</t>
@@ -7609,18 +7745,18 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>typing</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="28.05" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>vocab.viola</t>
@@ -7641,10 +7777,10 @@
           <t>adj</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
           <t>unveränderlich</t>
@@ -7656,7 +7792,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -7668,7 +7804,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="28.05" customHeight="1">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
@@ -7680,7 +7816,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="28.05" customHeight="1">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -7692,7 +7828,7 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="28.05" customHeight="1">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
@@ -7704,7 +7840,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="17.4" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>SÄTZE</t>
@@ -7745,7 +7881,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="28.05" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>La mia macchina è rossa.</t>
@@ -7756,9 +7892,9 @@
           <t>Mein Auto ist rot.</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+      <c r="C25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="28.05" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Il cielo è blu e l'erba è verde.</t>
@@ -7769,9 +7905,9 @@
           <t>Der Himmel ist blau und das Gras ist grün.</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="28.05" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Ho una maglia bianca e nera.</t>
@@ -7782,14 +7918,14 @@
           <t>Ich habe ein weiß-schwarzes Shirt.</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
+      <c r="C27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="28.05" customHeight="1">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>

</xml_diff>